<commit_message>
Updated FRA_grids_kan25 model - 2026-07-24 19:08
</commit_message>
<xml_diff>
--- a/VerveStacks_FRA_grids_kan25/Sets-vervestacks.xlsx
+++ b/VerveStacks_FRA_grids_kan25/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_FRA_grids_kan25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DCB5F40C-49F1-495F-AA97-4AA1B3E39CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8F9134B-3C5E-40B6-A375-99926D4102FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -367,7 +367,7 @@
     <t>p_w24020601-400_FRA</t>
   </si>
   <si>
-    <t>e_w24020601-400_FRA*</t>
+    <t>*[_]w24020601-400_FRA</t>
   </si>
   <si>
     <t>OR</t>
@@ -376,151 +376,151 @@
     <t>p_w27259817-400_FRA</t>
   </si>
   <si>
-    <t>e_w27259817-400_FRA*</t>
+    <t>*[_]w27259817-400_FRA</t>
   </si>
   <si>
     <t>p_w36805588-400_FRA</t>
   </si>
   <si>
-    <t>e_w36805588-400_FRA*</t>
+    <t>*[_]w36805588-400_FRA</t>
   </si>
   <si>
     <t>p_w49510896-400_FRA</t>
   </si>
   <si>
-    <t>e_w49510896-400_FRA*</t>
+    <t>*[_]w49510896-400_FRA</t>
   </si>
   <si>
     <t>p_w71933077-400_FRA</t>
   </si>
   <si>
-    <t>e_w71933077-400_FRA*</t>
+    <t>*[_]w71933077-400_FRA</t>
   </si>
   <si>
     <t>p_w79866837-400_FRA</t>
   </si>
   <si>
-    <t>e_w79866837-400_FRA*</t>
+    <t>*[_]w79866837-400_FRA</t>
   </si>
   <si>
     <t>p_w81641090-400_FRA</t>
   </si>
   <si>
-    <t>e_w81641090-400_FRA*</t>
+    <t>*[_]w81641090-400_FRA</t>
   </si>
   <si>
     <t>p_w82599261-400_FRA</t>
   </si>
   <si>
-    <t>e_w82599261-400_FRA*</t>
+    <t>*[_]w82599261-400_FRA</t>
   </si>
   <si>
     <t>p_w82825438-400_FRA</t>
   </si>
   <si>
-    <t>e_w82825438-400_FRA*</t>
+    <t>*[_]w82825438-400_FRA</t>
   </si>
   <si>
     <t>p_w85047359-400_FRA</t>
   </si>
   <si>
-    <t>e_w85047359-400_FRA*</t>
+    <t>*[_]w85047359-400_FRA</t>
   </si>
   <si>
     <t>p_w85203486-400_FRA</t>
   </si>
   <si>
-    <t>e_w85203486-400_FRA*</t>
+    <t>*[_]w85203486-400_FRA</t>
   </si>
   <si>
     <t>p_w85605950-400_FRA</t>
   </si>
   <si>
-    <t>e_w85605950-400_FRA*</t>
+    <t>*[_]w85605950-400_FRA</t>
   </si>
   <si>
     <t>p_w85710783-400_FRA</t>
   </si>
   <si>
-    <t>e_w85710783-400_FRA*</t>
+    <t>*[_]w85710783-400_FRA</t>
   </si>
   <si>
     <t>p_w85995894-400_FRA</t>
   </si>
   <si>
-    <t>e_w85995894-400_FRA*</t>
+    <t>*[_]w85995894-400_FRA</t>
   </si>
   <si>
     <t>p_w90842395-400_FRA</t>
   </si>
   <si>
-    <t>e_w90842395-400_FRA*</t>
+    <t>*[_]w90842395-400_FRA</t>
   </si>
   <si>
     <t>p_w98890904-400_FRA</t>
   </si>
   <si>
-    <t>e_w98890904-400_FRA*</t>
+    <t>*[_]w98890904-400_FRA</t>
   </si>
   <si>
     <t>p_w99722046-400_FRA</t>
   </si>
   <si>
-    <t>e_w99722046-400_FRA*</t>
+    <t>*[_]w99722046-400_FRA</t>
   </si>
   <si>
     <t>p_w110086345-400_FRA</t>
   </si>
   <si>
-    <t>e_w110086345-400_FRA*</t>
+    <t>*[_]w110086345-400_FRA</t>
   </si>
   <si>
     <t>p_w111558550-400_FRA</t>
   </si>
   <si>
-    <t>e_w111558550-400_FRA*</t>
+    <t>*[_]w111558550-400_FRA</t>
   </si>
   <si>
     <t>p_w112342683-400_FRA</t>
   </si>
   <si>
-    <t>e_w112342683-400_FRA*</t>
+    <t>*[_]w112342683-400_FRA</t>
   </si>
   <si>
     <t>p_w118086309-400_FRA</t>
   </si>
   <si>
-    <t>e_w118086309-400_FRA*</t>
+    <t>*[_]w118086309-400_FRA</t>
   </si>
   <si>
     <t>p_w146695955-400_FRA</t>
   </si>
   <si>
-    <t>e_w146695955-400_FRA*</t>
+    <t>*[_]w146695955-400_FRA</t>
   </si>
   <si>
     <t>p_w147132694-400_FRA</t>
   </si>
   <si>
-    <t>e_w147132694-400_FRA*</t>
+    <t>*[_]w147132694-400_FRA</t>
   </si>
   <si>
     <t>p_w159167277-400_FRA</t>
   </si>
   <si>
-    <t>e_w159167277-400_FRA*</t>
+    <t>*[_]w159167277-400_FRA</t>
   </si>
   <si>
     <t>p_w179260933-400_FRA</t>
   </si>
   <si>
-    <t>e_w179260933-400_FRA*</t>
+    <t>*[_]w179260933-400_FRA</t>
   </si>
   <si>
     <t>p_w235370803-400_FRA</t>
   </si>
   <si>
-    <t>e_w235370803-400_FRA*</t>
+    <t>*[_]w235370803-400_FRA</t>
   </si>
   <si>
     <t>rez_spv_FRA_001</t>
@@ -1815,7 +1815,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705E1424-021B-4637-B053-C7567BE0E6AA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FC08A66-5353-4329-BFC3-6C5ABDB4C0B0}">
   <dimension ref="B9:E111"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>